<commit_message>
xl sheet template added
</commit_message>
<xml_diff>
--- a/static/artezo_bulk_product_template.xlsx
+++ b/static/artezo_bulk_product_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Artezo_Project\bulk_product_sheet_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFDB521-C925-4DB2-9803-0C514846F10F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ABBEF3E-786D-480F-9061-CCAA30529F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="230">
   <si>
     <t>REQUIRED</t>
   </si>
@@ -561,9 +561,6 @@
     <t>Index-aligned — blank if none for that step</t>
   </si>
   <si>
-    <t>4 columns are mandatory: product name, category, sku, current stock. Rows missing any of these are skipped with a clear message.</t>
-  </si>
-  <si>
     <t>SEMICOLONS</t>
   </si>
   <si>
@@ -652,6 +649,81 @@
   </si>
   <si>
     <t>ART-WPLATE-GLD;ART-WPLATE-BLKK</t>
+  </si>
+  <si>
+    <t>HSN CODE</t>
+  </si>
+  <si>
+    <r>
+      <t>VARIANT</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> WEIGHT</t>
+    </r>
+  </si>
+  <si>
+    <t>VARIANT LENGTH</t>
+  </si>
+  <si>
+    <t>VARIANT BREADTH</t>
+  </si>
+  <si>
+    <t>VARIANT HEIGHT</t>
+  </si>
+  <si>
+    <t>VARIANTS REQUIRED</t>
+  </si>
+  <si>
+    <t>WEIGHT</t>
+  </si>
+  <si>
+    <t>HEIGHT</t>
+  </si>
+  <si>
+    <t>LENGTH</t>
+  </si>
+  <si>
+    <t>BREADTH</t>
+  </si>
+  <si>
+    <t>2.5;2</t>
+  </si>
+  <si>
+    <t>10;12</t>
+  </si>
+  <si>
+    <t>15;18</t>
+  </si>
+  <si>
+    <t>20;24</t>
+  </si>
+  <si>
+    <t>banner-demo;banner2.jpg</t>
+  </si>
+  <si>
+    <t>hsn code</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>length</t>
+  </si>
+  <si>
+    <t>breadth</t>
+  </si>
+  <si>
+    <t>height</t>
+  </si>
+  <si>
+    <t>9 columns are mandatory: product name, category, sku, hsn code, weight, length, breadth, height, current stock. Rows missing any of these are skipped with a clear message.</t>
   </si>
 </sst>
 </file>
@@ -1355,47 +1427,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ11"/>
+  <dimension ref="A1:AZ11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="24" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
-    <col min="13" max="14" width="13" customWidth="1"/>
-    <col min="15" max="15" width="16" customWidth="1"/>
-    <col min="16" max="16" width="36" customWidth="1"/>
-    <col min="17" max="18" width="28" customWidth="1"/>
-    <col min="19" max="19" width="18" customWidth="1"/>
-    <col min="20" max="20" width="20" customWidth="1"/>
-    <col min="21" max="22" width="40" customWidth="1"/>
-    <col min="23" max="23" width="18" customWidth="1"/>
-    <col min="24" max="24" width="60" customWidth="1"/>
-    <col min="25" max="25" width="22" customWidth="1"/>
-    <col min="26" max="26" width="28" customWidth="1"/>
-    <col min="27" max="27" width="26" customWidth="1"/>
-    <col min="28" max="28" width="20" customWidth="1"/>
-    <col min="29" max="29" width="18" customWidth="1"/>
-    <col min="30" max="33" width="14" customWidth="1"/>
+    <col min="3" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="13" width="13" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="17" max="17" width="15" customWidth="1"/>
+    <col min="18" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="16" customWidth="1"/>
+    <col min="21" max="21" width="36" customWidth="1"/>
+    <col min="22" max="23" width="28" customWidth="1"/>
+    <col min="24" max="24" width="18" customWidth="1"/>
+    <col min="25" max="25" width="20" customWidth="1"/>
+    <col min="26" max="27" width="40" customWidth="1"/>
+    <col min="28" max="28" width="18" customWidth="1"/>
+    <col min="29" max="29" width="60" customWidth="1"/>
+    <col min="30" max="30" width="22" customWidth="1"/>
+    <col min="31" max="31" width="28" customWidth="1"/>
+    <col min="32" max="32" width="26" customWidth="1"/>
+    <col min="33" max="33" width="20" customWidth="1"/>
     <col min="34" max="34" width="18" customWidth="1"/>
-    <col min="35" max="35" width="14" customWidth="1"/>
-    <col min="36" max="36" width="24" customWidth="1"/>
-    <col min="37" max="37" width="32" customWidth="1"/>
-    <col min="38" max="38" width="24" customWidth="1"/>
-    <col min="39" max="39" width="28" customWidth="1"/>
-    <col min="40" max="41" width="36" customWidth="1"/>
-    <col min="42" max="42" width="22" customWidth="1"/>
-    <col min="43" max="43" width="18" customWidth="1"/>
+    <col min="35" max="38" width="14" customWidth="1"/>
+    <col min="39" max="39" width="18" customWidth="1"/>
+    <col min="40" max="40" width="14" customWidth="1"/>
+    <col min="41" max="45" width="24" customWidth="1"/>
+    <col min="46" max="46" width="32" customWidth="1"/>
+    <col min="47" max="47" width="24" customWidth="1"/>
+    <col min="48" max="48" width="28" customWidth="1"/>
+    <col min="49" max="50" width="36" customWidth="1"/>
+    <col min="51" max="51" width="22" customWidth="1"/>
+    <col min="52" max="52" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:52" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1408,86 +1480,86 @@
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>1</v>
+      <c r="E1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="V1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="W1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="X1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="Y1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="Z1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="AA1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="AB1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="Z1" s="6" t="s">
+      <c r="AE1" s="6" t="s">
         <v>5</v>
-      </c>
-      <c r="AA1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AB1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AD1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AE1" s="7" t="s">
-        <v>6</v>
       </c>
       <c r="AF1" s="7" t="s">
         <v>6</v>
@@ -1504,29 +1576,56 @@
       <c r="AJ1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AK1" s="8" t="s">
+      <c r="AK1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AL1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AM1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AN1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AO1" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="AP1" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="AQ1" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="AR1" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="AS1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AT1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="AL1" s="8" t="s">
+      <c r="AU1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="AM1" s="9" t="s">
+      <c r="AV1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="AN1" s="9" t="s">
+      <c r="AW1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="AO1" s="9" t="s">
+      <c r="AX1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="AP1" s="9" t="s">
+      <c r="AY1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="AQ1" s="9" t="s">
+      <c r="AZ1" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="36" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:52" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>9</v>
       </c>
@@ -1537,258 +1636,312 @@
         <v>11</v>
       </c>
       <c r="D2" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="I2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="J2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="K2" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="L2" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="M2" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="N2" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="O2" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="P2" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="Q2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="R2" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="S2" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="T2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="U2" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="V2" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="W2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="X2" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="T2" s="13" t="s">
+      <c r="Y2" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="U2" s="14" t="s">
+      <c r="Z2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="V2" s="14" t="s">
+      <c r="AA2" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="W2" s="14" t="s">
+      <c r="AB2" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="X2" s="14" t="s">
+      <c r="AC2" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="Y2" s="15" t="s">
+      <c r="AD2" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="Z2" s="15" t="s">
+      <c r="AE2" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="AA2" s="16" t="s">
+      <c r="AF2" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="AB2" s="16" t="s">
+      <c r="AG2" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="AC2" s="16" t="s">
+      <c r="AH2" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="AD2" s="16" t="s">
+      <c r="AI2" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="AE2" s="16" t="s">
+      <c r="AJ2" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="AF2" s="16" t="s">
+      <c r="AK2" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="AG2" s="16" t="s">
+      <c r="AL2" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="AH2" s="16" t="s">
+      <c r="AM2" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AI2" s="16" t="s">
+      <c r="AN2" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="AJ2" s="16" t="s">
+      <c r="AO2" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="AP2" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="AQ2" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="AR2" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="AS2" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="AK2" s="17" t="s">
+      <c r="AT2" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="AL2" s="17" t="s">
+      <c r="AU2" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="AM2" s="18" t="s">
+      <c r="AV2" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="AN2" s="18" t="s">
+      <c r="AW2" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="AO2" s="18" t="s">
+      <c r="AX2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="AP2" s="18" t="s">
+      <c r="AY2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="AQ2" s="18" t="s">
+      <c r="AZ2" s="18" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:43" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:52" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="50" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="50" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C3" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="50">
+        <v>441122</v>
+      </c>
+      <c r="E3" s="50">
+        <v>2.6</v>
+      </c>
+      <c r="F3" s="50">
+        <v>10</v>
+      </c>
+      <c r="G3" s="50">
+        <v>15</v>
+      </c>
+      <c r="H3" s="50">
+        <v>20</v>
+      </c>
+      <c r="I3" s="50" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="J3" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="K3" s="50" t="s">
         <v>56</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="L3" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="M3" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="N3" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="J3" s="50" t="s">
+      <c r="O3" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="K3" s="50" t="s">
+      <c r="P3" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="L3" s="50" t="s">
+      <c r="Q3" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="M3" s="50" t="s">
+      <c r="R3" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="N3" s="50" t="s">
+      <c r="S3" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="O3" s="50" t="s">
+      <c r="T3" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="P3" s="50" t="s">
+      <c r="U3" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="Q3" s="50" t="s">
+      <c r="V3" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="R3" s="50" t="s">
+      <c r="W3" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="S3" s="50" t="s">
+      <c r="X3" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="T3" s="50" t="s">
+      <c r="Y3" s="50" t="s">
         <v>67</v>
       </c>
-      <c r="U3" s="50" t="s">
+      <c r="Z3" s="50" t="s">
         <v>68</v>
       </c>
-      <c r="V3" s="50" t="s">
+      <c r="AA3" s="50" t="s">
         <v>69</v>
       </c>
-      <c r="W3" s="50" t="s">
+      <c r="AB3" s="50" t="s">
         <v>70</v>
       </c>
-      <c r="X3" s="50" t="s">
+      <c r="AC3" s="50" t="s">
         <v>71</v>
       </c>
-      <c r="Y3" s="50" t="s">
+      <c r="AD3" s="50" t="s">
+        <v>206</v>
+      </c>
+      <c r="AE3" s="50" t="s">
         <v>207</v>
       </c>
-      <c r="Z3" s="50" t="s">
+      <c r="AF3" s="50" t="s">
         <v>208</v>
       </c>
-      <c r="AA3" s="50" t="s">
-        <v>209</v>
-      </c>
-      <c r="AB3" s="50" t="s">
+      <c r="AG3" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="AC3" s="50" t="s">
+      <c r="AH3" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="AD3" s="50" t="s">
+      <c r="AI3" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="AE3" s="50" t="s">
+      <c r="AJ3" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="AF3" s="50" t="s">
+      <c r="AK3" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="AG3" s="50" t="s">
+      <c r="AL3" s="50" t="s">
         <v>80</v>
       </c>
-      <c r="AH3" s="50" t="s">
+      <c r="AM3" s="50" t="s">
         <v>81</v>
       </c>
-      <c r="AI3" s="50" t="s">
+      <c r="AN3" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="AJ3" s="50" t="s">
+      <c r="AO3" s="50" t="s">
+        <v>219</v>
+      </c>
+      <c r="AP3" s="50" t="s">
+        <v>220</v>
+      </c>
+      <c r="AQ3" s="50" t="s">
+        <v>221</v>
+      </c>
+      <c r="AR3" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="AS3" s="50" t="s">
         <v>83</v>
       </c>
-      <c r="AK3" s="50" t="s">
+      <c r="AT3" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="AL3" s="50" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM3" s="50" t="s">
+      <c r="AU3" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="AV3" s="50" t="s">
         <v>86</v>
       </c>
-      <c r="AN3" s="50" t="s">
+      <c r="AW3" s="50" t="s">
         <v>87</v>
       </c>
-      <c r="AO3" s="50" t="s">
+      <c r="AX3" s="50" t="s">
         <v>88</v>
       </c>
-      <c r="AP3" s="50" t="s">
+      <c r="AY3" s="50" t="s">
         <v>89</v>
       </c>
-      <c r="AQ3" s="50" t="s">
+      <c r="AZ3" s="50" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:43" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:52" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="50"/>
       <c r="B4" s="50"/>
       <c r="C4" s="50"/>
@@ -1832,8 +1985,17 @@
       <c r="AO4" s="50"/>
       <c r="AP4" s="50"/>
       <c r="AQ4" s="50"/>
-    </row>
-    <row r="5" spans="1:43" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AR4" s="50"/>
+      <c r="AS4" s="50"/>
+      <c r="AT4" s="50"/>
+      <c r="AU4" s="50"/>
+      <c r="AV4" s="50"/>
+      <c r="AW4" s="50"/>
+      <c r="AX4" s="50"/>
+      <c r="AY4" s="50"/>
+      <c r="AZ4" s="50"/>
+    </row>
+    <row r="5" spans="1:52" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="50"/>
       <c r="B5" s="50"/>
       <c r="C5" s="50"/>
@@ -1877,8 +2039,17 @@
       <c r="AO5" s="50"/>
       <c r="AP5" s="50"/>
       <c r="AQ5" s="50"/>
-    </row>
-    <row r="6" spans="1:43" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AR5" s="50"/>
+      <c r="AS5" s="50"/>
+      <c r="AT5" s="50"/>
+      <c r="AU5" s="50"/>
+      <c r="AV5" s="50"/>
+      <c r="AW5" s="50"/>
+      <c r="AX5" s="50"/>
+      <c r="AY5" s="50"/>
+      <c r="AZ5" s="50"/>
+    </row>
+    <row r="6" spans="1:52" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="50"/>
       <c r="B6" s="50"/>
       <c r="C6" s="50"/>
@@ -1922,8 +2093,17 @@
       <c r="AO6" s="50"/>
       <c r="AP6" s="50"/>
       <c r="AQ6" s="50"/>
-    </row>
-    <row r="7" spans="1:43" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AR6" s="50"/>
+      <c r="AS6" s="50"/>
+      <c r="AT6" s="50"/>
+      <c r="AU6" s="50"/>
+      <c r="AV6" s="50"/>
+      <c r="AW6" s="50"/>
+      <c r="AX6" s="50"/>
+      <c r="AY6" s="50"/>
+      <c r="AZ6" s="50"/>
+    </row>
+    <row r="7" spans="1:52" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="50"/>
       <c r="B7" s="50"/>
       <c r="C7" s="50"/>
@@ -1967,8 +2147,17 @@
       <c r="AO7" s="50"/>
       <c r="AP7" s="50"/>
       <c r="AQ7" s="50"/>
-    </row>
-    <row r="8" spans="1:43" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AR7" s="50"/>
+      <c r="AS7" s="50"/>
+      <c r="AT7" s="50"/>
+      <c r="AU7" s="50"/>
+      <c r="AV7" s="50"/>
+      <c r="AW7" s="50"/>
+      <c r="AX7" s="50"/>
+      <c r="AY7" s="50"/>
+      <c r="AZ7" s="50"/>
+    </row>
+    <row r="8" spans="1:52" s="49" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="50"/>
       <c r="B8" s="50"/>
       <c r="C8" s="50"/>
@@ -2012,8 +2201,17 @@
       <c r="AO8" s="50"/>
       <c r="AP8" s="50"/>
       <c r="AQ8" s="50"/>
-    </row>
-    <row r="9" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AR8" s="50"/>
+      <c r="AS8" s="50"/>
+      <c r="AT8" s="50"/>
+      <c r="AU8" s="50"/>
+      <c r="AV8" s="50"/>
+      <c r="AW8" s="50"/>
+      <c r="AX8" s="50"/>
+      <c r="AY8" s="50"/>
+      <c r="AZ8" s="50"/>
+    </row>
+    <row r="9" spans="1:52" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="20"/>
       <c r="B9" s="20"/>
       <c r="C9" s="20"/>
@@ -2057,8 +2255,17 @@
       <c r="AO9" s="20"/>
       <c r="AP9" s="20"/>
       <c r="AQ9" s="20"/>
-    </row>
-    <row r="10" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AR9" s="20"/>
+      <c r="AS9" s="20"/>
+      <c r="AT9" s="20"/>
+      <c r="AU9" s="20"/>
+      <c r="AV9" s="20"/>
+      <c r="AW9" s="20"/>
+      <c r="AX9" s="20"/>
+      <c r="AY9" s="20"/>
+      <c r="AZ9" s="20"/>
+    </row>
+    <row r="10" spans="1:52" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="19"/>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
@@ -2102,13 +2309,22 @@
       <c r="AO10" s="19"/>
       <c r="AP10" s="19"/>
       <c r="AQ10" s="19"/>
-    </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="AR10" s="19"/>
+      <c r="AS10" s="19"/>
+      <c r="AT10" s="19"/>
+      <c r="AU10" s="19"/>
+      <c r="AV10" s="19"/>
+      <c r="AW10" s="19"/>
+      <c r="AX10" s="19"/>
+      <c r="AY10" s="19"/>
+      <c r="AZ10" s="19"/>
+    </row>
+    <row r="11" spans="1:52" x14ac:dyDescent="0.35">
       <c r="B11" s="49"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="K9:O1000" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="P9:T1000" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"true,false,yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2119,7 +2335,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2194,7 +2410,7 @@
         <v>100</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F4" s="24" t="s">
         <v>103</v>
@@ -2222,7 +2438,7 @@
     </row>
     <row r="6" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="22" t="s">
-        <v>105</v>
+        <v>224</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>99</v>
@@ -2233,790 +2449,890 @@
       <c r="D6" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="24" t="s">
-        <v>54</v>
+      <c r="E6" s="24">
+        <v>441122</v>
       </c>
       <c r="F6" s="24" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="E7" s="24">
+        <v>2.6</v>
+      </c>
+      <c r="F7" s="24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="25" t="s">
+    <row r="8" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="22" t="s">
+        <v>226</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="E8" s="24">
+        <v>10</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="22" t="s">
+        <v>227</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="24">
+        <v>15</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="E10" s="24">
+        <v>20</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="24">
+        <v>150</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="B7" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C7" s="27" t="s">
+      <c r="B12" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D12" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E12" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="F7" s="28" t="s">
+      <c r="F12" s="28" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="29" t="s">
+    <row r="13" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="B8" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C8" s="31" t="s">
+      <c r="B13" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D13" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E13" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F13" s="32" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="25" t="s">
+    <row r="14" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="B9" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" s="27" t="s">
+      <c r="B14" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D14" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="E9" s="28" t="s">
+      <c r="E14" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F14" s="28" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="29" t="s">
+    <row r="15" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="B10" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C10" s="31" t="s">
+      <c r="B15" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="D15" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="E10" s="32" t="s">
+      <c r="E15" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F15" s="32" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="25" t="s">
+    <row r="16" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C11" s="27" t="s">
+      <c r="B16" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D11" s="28" t="s">
+      <c r="D16" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="E11" s="28" t="s">
+      <c r="E16" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F16" s="28" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="29" t="s">
+    <row r="17" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="B12" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C12" s="31" t="s">
+      <c r="B17" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="D17" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="E12" s="32" t="s">
+      <c r="E17" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="F12" s="32" t="s">
+      <c r="F17" s="32" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="25" t="s">
+    <row r="18" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="25" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C13" s="33" t="s">
+      <c r="B18" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="28" t="s">
+      <c r="D18" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="E13" s="28" t="s">
+      <c r="E18" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="F13" s="28" t="s">
+      <c r="F18" s="28" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="29" t="s">
+    <row r="19" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="29" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C14" s="34" t="s">
+      <c r="B19" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C19" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D19" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="E14" s="32" t="s">
+      <c r="E19" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="F14" s="32" t="s">
+      <c r="F19" s="32" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="25" t="s">
+    <row r="20" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="B15" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C15" s="33" t="s">
+      <c r="B20" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="28" t="s">
+      <c r="D20" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="E15" s="28" t="s">
+      <c r="E20" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="F15" s="28" t="s">
+      <c r="F20" s="28" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="29" t="s">
+    <row r="21" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="B16" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C16" s="34" t="s">
+      <c r="B21" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C21" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D21" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="E16" s="32" t="s">
+      <c r="E21" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="32" t="s">
+      <c r="F21" s="32" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="25" t="s">
+    <row r="22" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C17" s="33" t="s">
+      <c r="B22" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D22" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E22" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F22" s="28" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="29" t="s">
+    <row r="23" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C18" s="35" t="s">
+      <c r="B23" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D23" s="32" t="s">
         <v>131</v>
       </c>
-      <c r="E18" s="32" t="s">
+      <c r="E23" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="F18" s="32" t="s">
+      <c r="F23" s="32" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="25" t="s">
+    <row r="24" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="B19" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C19" s="36" t="s">
+      <c r="B24" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C24" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="D19" s="28" t="s">
+      <c r="D24" s="28" t="s">
         <v>131</v>
       </c>
-      <c r="E19" s="28" t="s">
+      <c r="E24" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="F24" s="28" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="29" t="s">
+    <row r="25" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="29" t="s">
         <v>134</v>
       </c>
-      <c r="B20" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C20" s="35" t="s">
+      <c r="B25" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D25" s="32" t="s">
         <v>131</v>
       </c>
-      <c r="E20" s="32" t="s">
+      <c r="E25" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="F20" s="32" t="s">
+      <c r="F25" s="32" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="25" t="s">
+    <row r="26" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="B21" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C21" s="36" t="s">
+      <c r="B26" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="D21" s="28" t="s">
+      <c r="D26" s="28" t="s">
         <v>131</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E26" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="F21" s="28" t="s">
+      <c r="F26" s="28" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="29" t="s">
+    <row r="27" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="B22" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C22" s="35" t="s">
+      <c r="B27" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="32" t="s">
+      <c r="D27" s="32" t="s">
         <v>131</v>
       </c>
-      <c r="E22" s="32" t="s">
+      <c r="E27" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="F22" s="32" t="s">
+      <c r="F27" s="32" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="25" t="s">
+    <row r="28" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="B23" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C23" s="37" t="s">
+      <c r="B28" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="28" t="s">
+      <c r="D28" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E28" s="28" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="F28" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="29" t="s">
+    <row r="29" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="B24" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C24" s="38" t="s">
+      <c r="B29" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="D24" s="32" t="s">
+      <c r="D29" s="32" t="s">
         <v>139</v>
       </c>
-      <c r="E24" s="32" t="s">
+      <c r="E29" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="F24" s="32" t="s">
+      <c r="F29" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="25" t="s">
+    <row r="30" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="B25" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C25" s="37" t="s">
+      <c r="B30" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="D25" s="28" t="s">
+      <c r="D30" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="E25" s="28" t="s">
+      <c r="E30" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="F25" s="28" t="s">
+      <c r="F30" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="29" t="s">
+    <row r="31" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="29" t="s">
         <v>143</v>
       </c>
-      <c r="B26" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C26" s="38" t="s">
+      <c r="B31" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C31" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="D26" s="32" t="s">
+      <c r="D31" s="32" t="s">
         <v>139</v>
       </c>
-      <c r="E26" s="32" t="s">
+      <c r="E31" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="F26" s="32" t="s">
+      <c r="F31" s="32" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="25" t="s">
+    <row r="32" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="B27" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C27" s="39" t="s">
+      <c r="B32" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C32" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="D27" s="28" t="s">
+      <c r="D32" s="28" t="s">
         <v>146</v>
       </c>
-      <c r="E27" s="28" t="s">
+      <c r="E32" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="F27" s="28" t="s">
+      <c r="F32" s="28" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="29" t="s">
+    <row r="33" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="B28" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C28" s="40" t="s">
+      <c r="B33" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="D28" s="32" t="s">
+      <c r="D33" s="32" t="s">
         <v>146</v>
       </c>
-      <c r="E28" s="32" t="s">
+      <c r="E33" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F28" s="32" t="s">
+      <c r="F33" s="32" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="25" t="s">
+    <row r="34" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="25" t="s">
         <v>150</v>
       </c>
-      <c r="B29" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C29" s="41" t="s">
+      <c r="B34" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C34" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="28" t="s">
+      <c r="D34" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E29" s="28" t="s">
+      <c r="E34" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="F29" s="28" t="s">
+      <c r="F34" s="28" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="29" t="s">
+    <row r="35" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="B30" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C30" s="42" t="s">
+      <c r="B35" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D30" s="32" t="s">
+      <c r="D35" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E30" s="32" t="s">
+      <c r="E35" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="F30" s="32" t="s">
+      <c r="F35" s="32" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="25" t="s">
+    <row r="36" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="B31" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C31" s="41" t="s">
+      <c r="B36" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C36" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="D31" s="28" t="s">
+      <c r="D36" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E31" s="28" t="s">
+      <c r="E36" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="F31" s="28" t="s">
+      <c r="F36" s="28" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="29" t="s">
+    <row r="37" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="B32" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C32" s="42" t="s">
+      <c r="B37" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D32" s="32" t="s">
+      <c r="D37" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E32" s="32" t="s">
+      <c r="E37" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="F32" s="32" t="s">
+      <c r="F37" s="32" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="25" t="s">
+    <row r="38" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="B33" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C33" s="41" t="s">
+      <c r="B38" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C38" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="D33" s="28" t="s">
+      <c r="D38" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E33" s="28" t="s">
+      <c r="E38" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="F33" s="28" t="s">
+      <c r="F38" s="28" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="29" t="s">
+    <row r="39" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="B34" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C34" s="42" t="s">
+      <c r="B39" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C39" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D34" s="32" t="s">
+      <c r="D39" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E34" s="32" t="s">
+      <c r="E39" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="F34" s="32" t="s">
+      <c r="F39" s="32" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="25" t="s">
+    <row r="40" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="25" t="s">
         <v>161</v>
       </c>
-      <c r="B35" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C35" s="41" t="s">
+      <c r="B40" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C40" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="D35" s="28" t="s">
+      <c r="D40" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E35" s="28" t="s">
+      <c r="E40" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="F35" s="28" t="s">
+      <c r="F40" s="28" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="29" t="s">
+    <row r="41" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="B36" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C36" s="42" t="s">
+      <c r="B41" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C41" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D36" s="32" t="s">
+      <c r="D41" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E36" s="32" t="s">
+      <c r="E41" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="F36" s="32" t="s">
+      <c r="F41" s="32" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="25" t="s">
+    <row r="42" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="B37" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C37" s="41" t="s">
+      <c r="B42" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="D37" s="28" t="s">
+      <c r="D42" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E37" s="28" t="s">
+      <c r="E42" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="F37" s="28" t="s">
+      <c r="F42" s="28" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="29" t="s">
+    <row r="43" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="29" t="s">
         <v>166</v>
       </c>
-      <c r="B38" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C38" s="42" t="s">
+      <c r="B43" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C43" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D38" s="32" t="s">
+      <c r="D43" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E38" s="32" t="s">
+      <c r="E43" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="F38" s="32" t="s">
+      <c r="F43" s="32" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="25" t="s">
+    <row r="44" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="B39" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C39" s="43" t="s">
+      <c r="B44" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C44" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="D39" s="28" t="s">
+      <c r="D44" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E39" s="28" t="s">
+      <c r="E44" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="F39" s="28" t="s">
+      <c r="F44" s="28" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="29" t="s">
+    <row r="45" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="29" t="s">
         <v>170</v>
       </c>
-      <c r="B40" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C40" s="44" t="s">
+      <c r="B45" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C45" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="D40" s="32" t="s">
+      <c r="D45" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E40" s="32" t="s">
+      <c r="E45" s="32" t="s">
         <v>85</v>
       </c>
-      <c r="F40" s="32" t="s">
+      <c r="F45" s="32" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="25" t="s">
+    <row r="46" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="B41" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C41" s="45" t="s">
+      <c r="B46" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="D41" s="28" t="s">
+      <c r="D46" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E41" s="28" t="s">
+      <c r="E46" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="F41" s="28" t="s">
+      <c r="F46" s="28" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="29" t="s">
+    <row r="47" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="29" t="s">
         <v>173</v>
       </c>
-      <c r="B42" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C42" s="46" t="s">
+      <c r="B47" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C47" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="D42" s="32" t="s">
+      <c r="D47" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E42" s="32" t="s">
+      <c r="E47" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="F42" s="32" t="s">
+      <c r="F47" s="32" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="25" t="s">
+    <row r="48" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="B43" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C43" s="45" t="s">
+      <c r="B48" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C48" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="D43" s="28" t="s">
+      <c r="D48" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E43" s="28" t="s">
+      <c r="E48" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="F43" s="28" t="s">
+      <c r="F48" s="28" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="29" t="s">
+    <row r="49" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="29" t="s">
         <v>176</v>
       </c>
-      <c r="B44" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="C44" s="46" t="s">
+      <c r="B49" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C49" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="D44" s="32" t="s">
+      <c r="D49" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E44" s="32" t="s">
+      <c r="E49" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="F44" s="32" t="s">
+      <c r="F49" s="32" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="25" t="s">
+    <row r="50" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="B45" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C45" s="45" t="s">
+      <c r="B50" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C50" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="D45" s="28" t="s">
+      <c r="D50" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="E45" s="28" t="s">
+      <c r="E50" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="F45" s="28" t="s">
+      <c r="F50" s="28" t="s">
         <v>178</v>
       </c>
     </row>
@@ -3039,7 +3355,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B1" s="52"/>
     </row>
@@ -3048,23 +3364,23 @@
         <v>0</v>
       </c>
       <c r="B2" s="47" t="s">
-        <v>179</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B3" s="48" t="s">
         <v>180</v>
-      </c>
-      <c r="B3" s="48" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B4" s="47" t="s">
         <v>182</v>
-      </c>
-      <c r="B4" s="47" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
@@ -3072,7 +3388,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="48" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
@@ -3080,7 +3396,7 @@
         <v>44</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
@@ -3088,7 +3404,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="48" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
@@ -3096,7 +3412,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="47" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
@@ -3104,71 +3420,71 @@
         <v>51</v>
       </c>
       <c r="B9" s="48" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="B10" s="47" t="s">
         <v>189</v>
-      </c>
-      <c r="B10" s="47" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B11" s="48" t="s">
         <v>191</v>
-      </c>
-      <c r="B11" s="48" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="B12" s="47" t="s">
         <v>193</v>
-      </c>
-      <c r="B12" s="47" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="B13" s="48" t="s">
         <v>195</v>
-      </c>
-      <c r="B13" s="48" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="B14" s="47" t="s">
         <v>197</v>
-      </c>
-      <c r="B14" s="47" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="B15" s="48" t="s">
         <v>199</v>
-      </c>
-      <c r="B15" s="48" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="B16" s="47" t="s">
         <v>201</v>
-      </c>
-      <c r="B16" s="47" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="B17" s="48" t="s">
         <v>203</v>
-      </c>
-      <c r="B17" s="48" t="s">
-        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>